<commit_message>
feat: carga inicial Nivel 3 — Repuestos Autos y Camionetas (22 categorías)
Accesorios para Vehículos > Repuestos Autos y Camionetas > [22 subcategorías]
Fuente: captura de pantalla árbol MeLi AR
</commit_message>
<xml_diff>
--- a/categorias_autopartes_meli.xlsx
+++ b/categorias_autopartes_meli.xlsx
@@ -490,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -547,22 +547,459 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Autopartes y Accesorios</t>
+          <t>Repuestos Autos y Camionetas</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>TEST</t>
+          <t>Baterías</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr"/>
       <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="6" t="inlineStr"/>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>Fila de prueba — reemplazar con datos reales</t>
-        </is>
-      </c>
+      <c r="G2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Cerraduras y Llaves</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Climatización</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Componentes de Seguridad</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Conducción Asistida Avanzada</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Electroventiladores</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr"/>
+      <c r="G8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Eléctricos, Híbridos y PHEV</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr"/>
+      <c r="E9" s="5" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Encendido</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Filtros</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr"/>
+      <c r="G12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Frenos</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr"/>
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Iluminación</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="G14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Instalaciones Eléctricas</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr"/>
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Inyección</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr"/>
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr"/>
+      <c r="G16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Motor</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr"/>
+      <c r="E17" s="5" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr"/>
+      <c r="G17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="5" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Repuestos de Exterior</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr"/>
+      <c r="E19" s="5" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr"/>
+      <c r="G19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Repuestos de Habitáculo</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr"/>
+      <c r="G20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Suspensión y Dirección</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="5" t="inlineStr"/>
+      <c r="F21" s="6" t="inlineStr"/>
+      <c r="G21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Transmisión</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr"/>
+      <c r="G22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Ventanas y Sellos</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="5" t="inlineStr"/>
+      <c r="F23" s="6" t="inlineStr"/>
+      <c r="G23" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>

</xml_diff>

<commit_message>
feat: Baterías marcada como categoría terminal (sin N4)
Verificado via captura: va directo a productos sin subcategorías
</commit_message>
<xml_diff>
--- a/categorias_autopartes_meli.xlsx
+++ b/categorias_autopartes_meli.xlsx
@@ -558,7 +558,11 @@
       <c r="D2" s="5" t="inlineStr"/>
       <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="6" t="inlineStr"/>
-      <c r="G2" s="7" t="inlineStr"/>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Categoría terminal — sin subcategorías (va directo a productos)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat: add URL_Categoria column + Carrocería N4 (37 subcategorías)
- Nueva columna URL_Categoria con patrón verificado desde screenshot
- url_n3() / url_n4() helpers para construir URLs por slug
- Carrocería expandida a 37 filas N4 (URL N3 verificada ✓)
- Baterías: URL inferida por slug (*)
- 20 categorías N3 marcadas como "Pendiente captura N4"
- Output report: totales completas vs pendientes
</commit_message>
<xml_diff>
--- a/categorias_autopartes_meli.xlsx
+++ b/categorias_autopartes_meli.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Categorias MeLi AR" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Categorias MeLi AR'!$A$1:$G$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Categorias MeLi AR'!$A$1:$H$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,7 +33,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0F2FE"/>
       </patternFill>
     </fill>
     <fill>
@@ -102,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -123,6 +128,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -490,16 +498,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="70" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -530,10 +539,15 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>URL_Categoria</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>ID_Categoria_MLA</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -557,10 +571,15 @@
       </c>
       <c r="D2" s="5" t="inlineStr"/>
       <c r="E2" s="5" t="inlineStr"/>
-      <c r="F2" s="6" t="inlineStr"/>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>Categoría terminal — sin subcategorías (va directo a productos)</t>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/baterias/</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr"/>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>* URL inferida | Terminal — va directo a productos</t>
         </is>
       </c>
     </row>
@@ -580,10 +599,19 @@
           <t>Carrocería</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Alojamientos de Ópticas</t>
+        </is>
+      </c>
       <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="6" t="inlineStr"/>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="8" t="inlineStr"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -598,13 +626,22 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Cerraduras y Llaves</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Barras</t>
+        </is>
+      </c>
       <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -619,13 +656,22 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Climatización</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Baúles</t>
+        </is>
+      </c>
       <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="8" t="inlineStr"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -640,13 +686,22 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Componentes de Seguridad</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Baúles y Tapas Traseras</t>
+        </is>
+      </c>
       <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -661,13 +716,22 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Conducción Asistida Avanzada</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Bisagras</t>
+        </is>
+      </c>
       <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="8" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -682,13 +746,22 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Electroventiladores</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Capot</t>
+        </is>
+      </c>
       <c r="E8" s="5" t="inlineStr"/>
-      <c r="F8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G8" s="7" t="inlineStr"/>
+      <c r="H8" s="8" t="inlineStr"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -703,13 +776,22 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Eléctricos, Híbridos y PHEV</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Cerraduras</t>
+        </is>
+      </c>
       <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G9" s="7" t="inlineStr"/>
+      <c r="H9" s="8" t="inlineStr"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -724,13 +806,22 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Encendido</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Componentes Adicionales</t>
+        </is>
+      </c>
       <c r="E10" s="5" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G10" s="7" t="inlineStr"/>
+      <c r="H10" s="8" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -745,13 +836,22 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Escapes</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Espejos Retrovisores y Vidrios</t>
+        </is>
+      </c>
       <c r="E11" s="5" t="inlineStr"/>
-      <c r="F11" s="6" t="inlineStr"/>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G11" s="7" t="inlineStr"/>
+      <c r="H11" s="8" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -766,13 +866,22 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Filtros</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Grampas</t>
+        </is>
+      </c>
       <c r="E12" s="5" t="inlineStr"/>
-      <c r="F12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G12" s="7" t="inlineStr"/>
+      <c r="H12" s="8" t="inlineStr"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -787,13 +896,22 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Frenos</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Guardabarros</t>
+        </is>
+      </c>
       <c r="E13" s="5" t="inlineStr"/>
-      <c r="F13" s="6" t="inlineStr"/>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G13" s="7" t="inlineStr"/>
+      <c r="H13" s="8" t="inlineStr"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -808,13 +926,22 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Iluminación</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Laterales de Carrocería</t>
+        </is>
+      </c>
       <c r="E14" s="5" t="inlineStr"/>
-      <c r="F14" s="6" t="inlineStr"/>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G14" s="7" t="inlineStr"/>
+      <c r="H14" s="8" t="inlineStr"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -829,13 +956,22 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Instalaciones Eléctricas</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Manijas</t>
+        </is>
+      </c>
       <c r="E15" s="5" t="inlineStr"/>
-      <c r="F15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="8" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -850,13 +986,22 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Inyección</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Molduras</t>
+        </is>
+      </c>
       <c r="E16" s="5" t="inlineStr"/>
-      <c r="F16" s="6" t="inlineStr"/>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G16" s="7" t="inlineStr"/>
+      <c r="H16" s="8" t="inlineStr"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -871,13 +1016,22 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Motor</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
       <c r="E17" s="5" t="inlineStr"/>
-      <c r="F17" s="6" t="inlineStr"/>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G17" s="7" t="inlineStr"/>
+      <c r="H17" s="8" t="inlineStr"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
@@ -892,13 +1046,22 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Otros</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Paneles</t>
+        </is>
+      </c>
       <c r="E18" s="5" t="inlineStr"/>
-      <c r="F18" s="6" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G18" s="7" t="inlineStr"/>
+      <c r="H18" s="8" t="inlineStr"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -913,13 +1076,22 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Repuestos de Exterior</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Paneles de Cuarto</t>
+        </is>
+      </c>
       <c r="E19" s="5" t="inlineStr"/>
-      <c r="F19" s="6" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G19" s="7" t="inlineStr"/>
+      <c r="H19" s="8" t="inlineStr"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -934,13 +1106,22 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Repuestos de Habitáculo</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Paneles del Parabrisas</t>
+        </is>
+      </c>
       <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="6" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G20" s="7" t="inlineStr"/>
+      <c r="H20" s="8" t="inlineStr"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -955,13 +1136,22 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Suspensión y Dirección</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Paragolpes</t>
+        </is>
+      </c>
       <c r="E21" s="5" t="inlineStr"/>
-      <c r="F21" s="6" t="inlineStr"/>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G21" s="7" t="inlineStr"/>
+      <c r="H21" s="8" t="inlineStr"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -976,13 +1166,22 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Transmisión</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr"/>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Parrillas</t>
+        </is>
+      </c>
       <c r="E22" s="5" t="inlineStr"/>
-      <c r="F22" s="6" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
       <c r="G22" s="7" t="inlineStr"/>
+      <c r="H22" s="8" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
@@ -997,16 +1196,1025 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Pasaruedas</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr"/>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr"/>
+      <c r="H23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Pernos</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr"/>
+      <c r="H24" s="8" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Pilares</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr"/>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr"/>
+      <c r="H25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Pisos</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr"/>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr"/>
+      <c r="H26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Puertas y Paneles</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr"/>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr"/>
+      <c r="H27" s="8" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Rejillas para Faros Auxiliares</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr"/>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr"/>
+      <c r="H28" s="8" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Reparación de Cajas</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr"/>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr"/>
+      <c r="H29" s="8" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Soportes Elevación del Capó</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr"/>
+      <c r="H30" s="8" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Soportes de Rueda de Auxilio</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr"/>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr"/>
+      <c r="H31" s="8" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Soportes y Abrazaderas</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr"/>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr"/>
+      <c r="H32" s="8" t="inlineStr"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Tanques de Combustible</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr"/>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr"/>
+      <c r="H33" s="8" t="inlineStr"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Techos</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G34" s="7" t="inlineStr"/>
+      <c r="H34" s="8" t="inlineStr"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Techos Corredizos y Motores</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr"/>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr"/>
+      <c r="H35" s="8" t="inlineStr"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Tomas de Aire</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr"/>
+      <c r="H36" s="8" t="inlineStr"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Varillas de Apoyo</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr"/>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr"/>
+      <c r="H37" s="8" t="inlineStr"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Ventilaciones</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr"/>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr"/>
+      <c r="H38" s="8" t="inlineStr"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Carrocería</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Zócalos</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr"/>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr"/>
+      <c r="H39" s="8" t="inlineStr"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Cerraduras y Llaves</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr"/>
+      <c r="E40" s="5" t="inlineStr"/>
+      <c r="F40" s="6" t="inlineStr"/>
+      <c r="G40" s="7" t="inlineStr"/>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Climatización</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr"/>
+      <c r="E41" s="5" t="inlineStr"/>
+      <c r="F41" s="6" t="inlineStr"/>
+      <c r="G41" s="7" t="inlineStr"/>
+      <c r="H41" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Componentes de Seguridad</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr"/>
+      <c r="F42" s="6" t="inlineStr"/>
+      <c r="G42" s="7" t="inlineStr"/>
+      <c r="H42" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Conducción Asistida Avanzada</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr"/>
+      <c r="F43" s="6" t="inlineStr"/>
+      <c r="G43" s="7" t="inlineStr"/>
+      <c r="H43" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Electroventiladores</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="6" t="inlineStr"/>
+      <c r="G44" s="7" t="inlineStr"/>
+      <c r="H44" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Eléctricos, Híbridos y PHEV</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr"/>
+      <c r="E45" s="5" t="inlineStr"/>
+      <c r="F45" s="6" t="inlineStr"/>
+      <c r="G45" s="7" t="inlineStr"/>
+      <c r="H45" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Encendido</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr"/>
+      <c r="F46" s="6" t="inlineStr"/>
+      <c r="G46" s="7" t="inlineStr"/>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Escapes</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr"/>
+      <c r="E47" s="5" t="inlineStr"/>
+      <c r="F47" s="6" t="inlineStr"/>
+      <c r="G47" s="7" t="inlineStr"/>
+      <c r="H47" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Filtros</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr"/>
+      <c r="E48" s="5" t="inlineStr"/>
+      <c r="F48" s="6" t="inlineStr"/>
+      <c r="G48" s="7" t="inlineStr"/>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Frenos</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr"/>
+      <c r="E49" s="5" t="inlineStr"/>
+      <c r="F49" s="6" t="inlineStr"/>
+      <c r="G49" s="7" t="inlineStr"/>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Iluminación</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr"/>
+      <c r="E50" s="5" t="inlineStr"/>
+      <c r="F50" s="6" t="inlineStr"/>
+      <c r="G50" s="7" t="inlineStr"/>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Instalaciones Eléctricas</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr"/>
+      <c r="E51" s="5" t="inlineStr"/>
+      <c r="F51" s="6" t="inlineStr"/>
+      <c r="G51" s="7" t="inlineStr"/>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Inyección</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr"/>
+      <c r="E52" s="5" t="inlineStr"/>
+      <c r="F52" s="6" t="inlineStr"/>
+      <c r="G52" s="7" t="inlineStr"/>
+      <c r="H52" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Motor</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr"/>
+      <c r="E53" s="5" t="inlineStr"/>
+      <c r="F53" s="6" t="inlineStr"/>
+      <c r="G53" s="7" t="inlineStr"/>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr"/>
+      <c r="E54" s="5" t="inlineStr"/>
+      <c r="F54" s="6" t="inlineStr"/>
+      <c r="G54" s="7" t="inlineStr"/>
+      <c r="H54" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Repuestos de Exterior</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr"/>
+      <c r="E55" s="5" t="inlineStr"/>
+      <c r="F55" s="6" t="inlineStr"/>
+      <c r="G55" s="7" t="inlineStr"/>
+      <c r="H55" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Repuestos de Habitáculo</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr"/>
+      <c r="E56" s="5" t="inlineStr"/>
+      <c r="F56" s="6" t="inlineStr"/>
+      <c r="G56" s="7" t="inlineStr"/>
+      <c r="H56" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Suspensión y Dirección</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr"/>
+      <c r="E57" s="5" t="inlineStr"/>
+      <c r="F57" s="6" t="inlineStr"/>
+      <c r="G57" s="7" t="inlineStr"/>
+      <c r="H57" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Transmisión</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr"/>
+      <c r="E58" s="5" t="inlineStr"/>
+      <c r="F58" s="6" t="inlineStr"/>
+      <c r="G58" s="7" t="inlineStr"/>
+      <c r="H58" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Accesorios para Vehículos</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Repuestos Autos y Camionetas</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
           <t>Ventanas y Sellos</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr"/>
-      <c r="E23" s="5" t="inlineStr"/>
-      <c r="F23" s="6" t="inlineStr"/>
-      <c r="G23" s="7" t="inlineStr"/>
+      <c r="D59" s="5" t="inlineStr"/>
+      <c r="E59" s="5" t="inlineStr"/>
+      <c r="F59" s="6" t="inlineStr"/>
+      <c r="G59" s="7" t="inlineStr"/>
+      <c r="H59" s="8" t="inlineStr">
+        <is>
+          <t>Pendiente captura N4</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G1"/>
+  <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Carrocería > Alojamientos de Ópticas marcada como Terminal N4
URL N4 inferida por slug | va directo a productos sin N5
</commit_message>
<xml_diff>
--- a/categorias_autopartes_meli.xlsx
+++ b/categorias_autopartes_meli.xlsx
@@ -607,11 +607,15 @@
       <c r="E3" s="5" t="inlineStr"/>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/</t>
+          <t>https://listado.mercadolibre.com.ar/accesorios-vehiculos/repuestos-autos-camionetas/carroceria/alojamientos-opticas/</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="8" t="inlineStr"/>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>* URL inferida | Terminal N4</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">

</xml_diff>